<commit_message>
Adding SOD for ver
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst_Ver/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst_Ver/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst_Ver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE7BE0C6-0296-4E3E-B1FF-442284501A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B97AE1-C101-444B-8C76-F43B683EF118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="88">
   <si>
     <t>Steps</t>
   </si>
@@ -266,21 +266,6 @@
   </si>
   <si>
     <t>Hearst_Ver/ActivityData/VER_BILL_2026-07-31.xlsx</t>
-  </si>
-  <si>
-    <t>Hearst_Ver/ActivityData/VER_SOD_2026-08-31.xlsx</t>
-  </si>
-  <si>
-    <t>Hearst_Ver/ActivityData/VER_PSD_2026-08-31.xlsx</t>
-  </si>
-  <si>
-    <t>Hearst_Ver/ActivityData/VER_BILL_2026-08-31.xlsx</t>
-  </si>
-  <si>
-    <t>Hearst_Ver/ActivityData/VER_PSD_2026-09-30.xlsx</t>
-  </si>
-  <si>
-    <t>Hearst_Ver/ActivityData/VER_PSD_2026-10-31.xlsx</t>
   </si>
   <si>
     <t>MetricLevelLtd</t>
@@ -607,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -787,7 +772,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -1459,94 +1444,6 @@
       </c>
       <c r="C61" s="1">
         <v>46234</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>18</v>
-      </c>
-      <c r="B62" t="s">
-        <v>4</v>
-      </c>
-      <c r="C62" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>9</v>
-      </c>
-      <c r="B63" t="s">
-        <v>4</v>
-      </c>
-      <c r="C63" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>9</v>
-      </c>
-      <c r="B64" t="s">
-        <v>4</v>
-      </c>
-      <c r="C64" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>22</v>
-      </c>
-      <c r="B65" t="s">
-        <v>23</v>
-      </c>
-      <c r="C65" s="1">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>9</v>
-      </c>
-      <c r="B66" t="s">
-        <v>4</v>
-      </c>
-      <c r="C66" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>22</v>
-      </c>
-      <c r="B67" t="s">
-        <v>23</v>
-      </c>
-      <c r="C67" s="1">
-        <v>46295</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>9</v>
-      </c>
-      <c r="B68" t="s">
-        <v>4</v>
-      </c>
-      <c r="C68" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>22</v>
-      </c>
-      <c r="B69" t="s">
-        <v>23</v>
-      </c>
-      <c r="C69" s="1">
-        <v>46326</v>
       </c>
     </row>
   </sheetData>
@@ -1569,27 +1466,27 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1597,7 +1494,7 @@
         <v>20251231</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C3">
         <v>-2221.4331999999999</v>
@@ -1614,7 +1511,7 @@
         <v>20251231</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C4">
         <v>-2221.4331999999999</v>
@@ -1631,7 +1528,7 @@
         <v>20251231</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C5">
         <v>-2221.4331999999999</v>
@@ -1648,7 +1545,7 @@
         <v>20260131</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C6" s="4">
         <v>-12.491199999999999</v>
@@ -1667,7 +1564,7 @@
         <v>20260131</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C7" s="4">
         <v>-12.491199999999999</v>
@@ -1686,7 +1583,7 @@
         <v>20260131</v>
       </c>
       <c r="B8" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C8" s="4">
         <v>-12.491199999999999</v>
@@ -1705,7 +1602,7 @@
         <v>20260228</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C9" s="4">
         <v>-4772.7052000000003</v>
@@ -1724,7 +1621,7 @@
         <v>20260228</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C10" s="4">
         <v>-4772.7052000000003</v>
@@ -1743,7 +1640,7 @@
         <v>20260228</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C11" s="4">
         <v>-4772.7052000000003</v>

</xml_diff>

<commit_message>
Checking in test file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst_Ver/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst_Ver/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst_Ver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065CCBCF-12E8-4EDB-BB57-E9FB83F6EB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE3FC56-A6A8-4BD8-8B67-37FA0DE1F6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="88">
   <si>
     <t>Steps</t>
   </si>
@@ -488,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -638,6 +638,50 @@
       </c>
       <c r="C13" s="1">
         <v>45657</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="1">
+        <v>45688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checking in Ver case
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst_Ver/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst_Ver/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst_Ver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE3FC56-A6A8-4BD8-8B67-37FA0DE1F6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5226E40C-86BA-4D0B-92E1-40A91199C475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="88">
   <si>
     <t>Steps</t>
   </si>
@@ -488,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -682,6 +682,754 @@
       </c>
       <c r="C17" s="1">
         <v>45688</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="1">
+        <v>45716</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="1">
+        <v>45747</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="1">
+        <v>45777</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C32" s="1">
+        <v>45808</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="1">
+        <v>45838</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" s="1">
+        <v>45869</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" s="1">
+        <v>45900</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" t="s">
+        <v>23</v>
+      </c>
+      <c r="C48" s="1">
+        <v>45930</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>18</v>
+      </c>
+      <c r="B49" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" t="s">
+        <v>23</v>
+      </c>
+      <c r="C52" s="1">
+        <v>45961</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>18</v>
+      </c>
+      <c r="B53" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>22</v>
+      </c>
+      <c r="B56" t="s">
+        <v>23</v>
+      </c>
+      <c r="C56" s="1">
+        <v>45991</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>9</v>
+      </c>
+      <c r="B58" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>9</v>
+      </c>
+      <c r="B59" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" t="s">
+        <v>23</v>
+      </c>
+      <c r="C60" s="1">
+        <v>46022</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>22</v>
+      </c>
+      <c r="B63" t="s">
+        <v>23</v>
+      </c>
+      <c r="C63" s="1">
+        <v>46053</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>18</v>
+      </c>
+      <c r="B64" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>9</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>9</v>
+      </c>
+      <c r="B66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>22</v>
+      </c>
+      <c r="B67" t="s">
+        <v>23</v>
+      </c>
+      <c r="C67" s="1">
+        <v>46081</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>18</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>9</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>9</v>
+      </c>
+      <c r="B70" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>22</v>
+      </c>
+      <c r="B71" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71" s="1">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>18</v>
+      </c>
+      <c r="B72" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>9</v>
+      </c>
+      <c r="B73" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>9</v>
+      </c>
+      <c r="B74" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>22</v>
+      </c>
+      <c r="B75" t="s">
+        <v>23</v>
+      </c>
+      <c r="C75" s="1">
+        <v>46142</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>18</v>
+      </c>
+      <c r="B76" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>9</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>22</v>
+      </c>
+      <c r="B78" t="s">
+        <v>23</v>
+      </c>
+      <c r="C78" s="1">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>18</v>
+      </c>
+      <c r="B79" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>9</v>
+      </c>
+      <c r="B80" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>9</v>
+      </c>
+      <c r="B81" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>22</v>
+      </c>
+      <c r="B82" t="s">
+        <v>23</v>
+      </c>
+      <c r="C82" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>18</v>
+      </c>
+      <c r="B83" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>9</v>
+      </c>
+      <c r="B84" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>22</v>
+      </c>
+      <c r="B85" t="s">
+        <v>23</v>
+      </c>
+      <c r="C85" s="1">
+        <v>46234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>